<commit_message>
quelque modification sur laffichage des programmes par defauts
</commit_message>
<xml_diff>
--- a/resources/Programmes/Programmematernellepetitesection.xlsx
+++ b/resources/Programmes/Programmematernellepetitesection.xlsx
@@ -1,17 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\JEANNE\Desktop\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <bookViews>
+    <workbookView xWindow="0" yWindow="0" windowWidth="20490" windowHeight="7155"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="Feuille 1" sheetId="1" r:id="rId4"/>
+    <sheet name="Feuille 1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="42">
   <si>
     <t>Activité</t>
   </si>
@@ -122,33 +130,63 @@
   </si>
   <si>
     <t>Précision des gestes, patience, concentration</t>
+  </si>
+  <si>
+    <t>Mode_evaluation</t>
+  </si>
+  <si>
+    <t>Bareme</t>
+  </si>
+  <si>
+    <t>null</t>
+  </si>
+  <si>
+    <t>Type_exercices</t>
+  </si>
+  <si>
+    <t>leçons</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="4">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
     </font>
     <font>
-      <sz val="11.0"/>
+      <sz val="11"/>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="2">
@@ -156,45 +194,72 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
-    <border/>
+  <borders count="2">
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="8">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment vertical="bottom"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="3" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment shrinkToFit="0" vertical="bottom" wrapText="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -384,55 +449,76 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:AA9"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="25.140625" customWidth="1"/>
+    <col min="2" max="2" width="26.140625" customWidth="1"/>
+    <col min="3" max="5" width="23.85546875" customWidth="1"/>
+    <col min="6" max="6" width="26.85546875" customWidth="1"/>
+    <col min="7" max="7" width="24.42578125" customWidth="1"/>
+    <col min="8" max="8" width="23" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="7" t="s">
+        <v>41</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2"/>
-      <c r="G1" s="2"/>
-      <c r="H1" s="2"/>
-      <c r="I1" s="2"/>
-      <c r="J1" s="2"/>
-      <c r="K1" s="2"/>
-      <c r="L1" s="2"/>
-      <c r="M1" s="2"/>
-      <c r="N1" s="2"/>
-      <c r="O1" s="2"/>
-      <c r="P1" s="2"/>
-      <c r="Q1" s="2"/>
-      <c r="R1" s="2"/>
-      <c r="S1" s="2"/>
-      <c r="T1" s="2"/>
-      <c r="U1" s="2"/>
-      <c r="V1" s="2"/>
-      <c r="W1" s="2"/>
-      <c r="X1" s="2"/>
-      <c r="Y1" s="2"/>
+      <c r="H1" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="I1" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="J1" s="1"/>
+      <c r="K1" s="1"/>
+      <c r="L1" s="1"/>
+      <c r="M1" s="1"/>
+      <c r="N1" s="1"/>
+      <c r="O1" s="1"/>
+      <c r="P1" s="1"/>
+      <c r="Q1" s="1"/>
+      <c r="R1" s="1"/>
+      <c r="S1" s="1"/>
+      <c r="T1" s="1"/>
+      <c r="U1" s="1"/>
+      <c r="V1" s="1"/>
+      <c r="W1" s="1"/>
+      <c r="X1" s="1"/>
+      <c r="Y1" s="1"/>
+      <c r="Z1" s="1"/>
+      <c r="AA1" s="1"/>
     </row>
-    <row r="2">
-      <c r="A2" s="3" t="s">
+    <row r="2" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
         <v>5</v>
       </c>
       <c r="B2" s="4" t="s">
@@ -442,34 +528,44 @@
         <v>7</v>
       </c>
       <c r="D2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F2" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="G2" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
-      <c r="H2" s="2"/>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
-      <c r="N2" s="2"/>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
-      <c r="T2" s="2"/>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2"/>
+      <c r="H2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J2" s="1"/>
+      <c r="K2" s="1"/>
+      <c r="L2" s="1"/>
+      <c r="M2" s="1"/>
+      <c r="N2" s="1"/>
+      <c r="O2" s="1"/>
+      <c r="P2" s="1"/>
+      <c r="Q2" s="1"/>
+      <c r="R2" s="1"/>
+      <c r="S2" s="1"/>
+      <c r="T2" s="1"/>
+      <c r="U2" s="1"/>
+      <c r="V2" s="1"/>
+      <c r="W2" s="1"/>
+      <c r="X2" s="1"/>
+      <c r="Y2" s="1"/>
+      <c r="Z2" s="1"/>
+      <c r="AA2" s="1"/>
     </row>
-    <row r="3">
-      <c r="A3" s="3" t="s">
+    <row r="3" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
         <v>10</v>
       </c>
       <c r="B3" s="4" t="s">
@@ -479,34 +575,44 @@
         <v>12</v>
       </c>
       <c r="D3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E3" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="G3" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
-      <c r="N3" s="2"/>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="2"/>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
+      <c r="H3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
+      <c r="N3" s="1"/>
+      <c r="O3" s="1"/>
+      <c r="P3" s="1"/>
+      <c r="Q3" s="1"/>
+      <c r="R3" s="1"/>
+      <c r="S3" s="1"/>
+      <c r="T3" s="1"/>
+      <c r="U3" s="1"/>
+      <c r="V3" s="1"/>
+      <c r="W3" s="1"/>
+      <c r="X3" s="1"/>
+      <c r="Y3" s="1"/>
+      <c r="Z3" s="1"/>
+      <c r="AA3" s="1"/>
     </row>
-    <row r="4">
-      <c r="A4" s="3" t="s">
+    <row r="4" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="6" t="s">
         <v>15</v>
       </c>
       <c r="B4" s="4" t="s">
@@ -516,34 +622,44 @@
         <v>17</v>
       </c>
       <c r="D4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E4" s="4" t="s">
+      <c r="G4" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
-      <c r="H4" s="2"/>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
-      <c r="N4" s="2"/>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="2"/>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
+      <c r="H4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J4" s="1"/>
+      <c r="K4" s="1"/>
+      <c r="L4" s="1"/>
+      <c r="M4" s="1"/>
+      <c r="N4" s="1"/>
+      <c r="O4" s="1"/>
+      <c r="P4" s="1"/>
+      <c r="Q4" s="1"/>
+      <c r="R4" s="1"/>
+      <c r="S4" s="1"/>
+      <c r="T4" s="1"/>
+      <c r="U4" s="1"/>
+      <c r="V4" s="1"/>
+      <c r="W4" s="1"/>
+      <c r="X4" s="1"/>
+      <c r="Y4" s="1"/>
+      <c r="Z4" s="1"/>
+      <c r="AA4" s="1"/>
     </row>
-    <row r="5">
-      <c r="A5" s="3" t="s">
+    <row r="5" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="6" t="s">
         <v>19</v>
       </c>
       <c r="B5" s="4" t="s">
@@ -553,34 +669,44 @@
         <v>21</v>
       </c>
       <c r="D5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F5" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="G5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
-      <c r="H5" s="2"/>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
-      <c r="N5" s="2"/>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="2"/>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
+      <c r="H5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J5" s="1"/>
+      <c r="K5" s="1"/>
+      <c r="L5" s="1"/>
+      <c r="M5" s="1"/>
+      <c r="N5" s="1"/>
+      <c r="O5" s="1"/>
+      <c r="P5" s="1"/>
+      <c r="Q5" s="1"/>
+      <c r="R5" s="1"/>
+      <c r="S5" s="1"/>
+      <c r="T5" s="1"/>
+      <c r="U5" s="1"/>
+      <c r="V5" s="1"/>
+      <c r="W5" s="1"/>
+      <c r="X5" s="1"/>
+      <c r="Y5" s="1"/>
+      <c r="Z5" s="1"/>
+      <c r="AA5" s="1"/>
     </row>
-    <row r="6">
-      <c r="A6" s="3" t="s">
+    <row r="6" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A6" s="6" t="s">
         <v>22</v>
       </c>
       <c r="B6" s="4" t="s">
@@ -590,34 +716,44 @@
         <v>24</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F6" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="G6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
-      <c r="N6" s="2"/>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="2"/>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+      <c r="H6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J6" s="1"/>
+      <c r="K6" s="1"/>
+      <c r="L6" s="1"/>
+      <c r="M6" s="1"/>
+      <c r="N6" s="1"/>
+      <c r="O6" s="1"/>
+      <c r="P6" s="1"/>
+      <c r="Q6" s="1"/>
+      <c r="R6" s="1"/>
+      <c r="S6" s="1"/>
+      <c r="T6" s="1"/>
+      <c r="U6" s="1"/>
+      <c r="V6" s="1"/>
+      <c r="W6" s="1"/>
+      <c r="X6" s="1"/>
+      <c r="Y6" s="1"/>
+      <c r="Z6" s="1"/>
+      <c r="AA6" s="1"/>
     </row>
-    <row r="7">
-      <c r="A7" s="3" t="s">
+    <row r="7" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A7" s="6" t="s">
         <v>26</v>
       </c>
       <c r="B7" s="4" t="s">
@@ -627,34 +763,44 @@
         <v>28</v>
       </c>
       <c r="D7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E7" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="G7" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
-      <c r="N7" s="2"/>
-      <c r="O7" s="2"/>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="2"/>
-      <c r="U7" s="2"/>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
+      <c r="H7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J7" s="1"/>
+      <c r="K7" s="1"/>
+      <c r="L7" s="1"/>
+      <c r="M7" s="1"/>
+      <c r="N7" s="1"/>
+      <c r="O7" s="1"/>
+      <c r="P7" s="1"/>
+      <c r="Q7" s="1"/>
+      <c r="R7" s="1"/>
+      <c r="S7" s="1"/>
+      <c r="T7" s="1"/>
+      <c r="U7" s="1"/>
+      <c r="V7" s="1"/>
+      <c r="W7" s="1"/>
+      <c r="X7" s="1"/>
+      <c r="Y7" s="1"/>
+      <c r="Z7" s="1"/>
+      <c r="AA7" s="1"/>
     </row>
-    <row r="8">
-      <c r="A8" s="3" t="s">
+    <row r="8" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A8" s="6" t="s">
         <v>30</v>
       </c>
       <c r="B8" s="4" t="s">
@@ -664,34 +810,44 @@
         <v>32</v>
       </c>
       <c r="D8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F8" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="G8" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
-      <c r="H8" s="2"/>
-      <c r="I8" s="2"/>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
-      <c r="N8" s="2"/>
-      <c r="O8" s="2"/>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="2"/>
-      <c r="U8" s="2"/>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
+      <c r="H8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I8" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J8" s="1"/>
+      <c r="K8" s="1"/>
+      <c r="L8" s="1"/>
+      <c r="M8" s="1"/>
+      <c r="N8" s="1"/>
+      <c r="O8" s="1"/>
+      <c r="P8" s="1"/>
+      <c r="Q8" s="1"/>
+      <c r="R8" s="1"/>
+      <c r="S8" s="1"/>
+      <c r="T8" s="1"/>
+      <c r="U8" s="1"/>
+      <c r="V8" s="1"/>
+      <c r="W8" s="1"/>
+      <c r="X8" s="1"/>
+      <c r="Y8" s="1"/>
+      <c r="Z8" s="1"/>
+      <c r="AA8" s="1"/>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="s">
+    <row r="9" spans="1:27" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A9" s="6" t="s">
         <v>34</v>
       </c>
       <c r="B9" s="4" t="s">
@@ -701,33 +857,44 @@
         <v>36</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="F9" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="G9" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
-      <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
-      <c r="N9" s="2"/>
-      <c r="O9" s="2"/>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="2"/>
-      <c r="U9" s="2"/>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
-      <c r="Y9" s="2"/>
+      <c r="H9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="I9" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="J9" s="1"/>
+      <c r="K9" s="1"/>
+      <c r="L9" s="1"/>
+      <c r="M9" s="1"/>
+      <c r="N9" s="1"/>
+      <c r="O9" s="1"/>
+      <c r="P9" s="1"/>
+      <c r="Q9" s="1"/>
+      <c r="R9" s="1"/>
+      <c r="S9" s="1"/>
+      <c r="T9" s="1"/>
+      <c r="U9" s="1"/>
+      <c r="V9" s="1"/>
+      <c r="W9" s="1"/>
+      <c r="X9" s="1"/>
+      <c r="Y9" s="1"/>
+      <c r="Z9" s="1"/>
+      <c r="AA9" s="1"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>